<commit_message>
Switch everything to Georgia and Calibri, remove slide pills, new photos
</commit_message>
<xml_diff>
--- a/pastoral-projects/the-planting-project/downloads/The_Planting_Project_Tracker.xlsx
+++ b/pastoral-projects/the-planting-project/downloads/The_Planting_Project_Tracker.xlsx
@@ -29,7 +29,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="dd\ mmm\ yyyy"/>
   </numFmts>
-  <fonts count="24">
+  <fonts count="32">
     <font>
       <name val="Calibri"/>
       <charset val="1"/>
@@ -128,60 +128,104 @@
       <sz val="9"/>
     </font>
     <font>
-      <name val="Libre Caslon Display"/>
+      <name val="Georgia"/>
       <b val="1"/>
       <color rgb="FF1F4E2C"/>
       <sz val="18"/>
     </font>
     <font>
-      <name val="Karla"/>
+      <name val="Calibri"/>
       <i val="1"/>
       <color rgb="FF8B9179"/>
       <sz val="10"/>
     </font>
     <font>
-      <name val="Libre Caslon Display"/>
+      <name val="Georgia"/>
       <b val="1"/>
       <color rgb="FF1F4E2C"/>
       <sz val="13"/>
     </font>
     <font>
-      <name val="Karla"/>
+      <name val="Calibri"/>
       <color rgb="FF1B2A1B"/>
       <sz val="11"/>
     </font>
     <font>
-      <name val="Libre Caslon Display"/>
+      <name val="Georgia"/>
       <b val="1"/>
       <color rgb="FF1F4E2C"/>
       <sz val="16"/>
     </font>
     <font>
-      <name val="Karla"/>
+      <name val="Calibri"/>
       <i val="1"/>
       <color rgb="FF8B9179"/>
       <sz val="9"/>
     </font>
     <font>
-      <name val="Karla"/>
+      <name val="Calibri"/>
       <b val="1"/>
       <color rgb="FF1F4E2C"/>
       <sz val="11"/>
     </font>
     <font>
-      <name val="Karla"/>
+      <name val="Calibri"/>
       <b val="1"/>
       <color rgb="FFFFFFFF"/>
       <sz val="11"/>
     </font>
     <font>
-      <name val="Karla"/>
+      <name val="Calibri"/>
       <i val="1"/>
       <color rgb="FF5B6B58"/>
       <sz val="10"/>
     </font>
     <font>
-      <name val="Karla"/>
+      <name val="Calibri"/>
+      <i val="1"/>
+      <color rgb="FFA3532A"/>
+      <sz val="9"/>
+    </font>
+    <font>
+      <name val="Georgia"/>
+      <color rgb="FF1F4E2C"/>
+      <sz val="18"/>
+    </font>
+    <font>
+      <name val="Georgia"/>
+      <color rgb="FF1F4E2C"/>
+      <sz val="13"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <color rgb="FF1B2A1B"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <name val="Georgia"/>
+      <color rgb="FF1F4E2C"/>
+      <sz val="16"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="FF1F4E2C"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="FFFFFFFF"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <i val="1"/>
+      <color rgb="FF5B6B58"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
       <i val="1"/>
       <color rgb="FFA3532A"/>
       <sz val="9"/>
@@ -285,7 +329,7 @@
     <xf numFmtId="42" fontId="3" fillId="0" borderId="0"/>
     <xf numFmtId="9" fontId="3" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="42">
+  <cellXfs count="50">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="general" vertical="bottom"/>
     </xf>
@@ -404,6 +448,30 @@
       <alignment horizontal="general" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="23" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="general" vertical="bottom"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="5" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="general" vertical="bottom"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="general" vertical="bottom"/>
+    </xf>
+    <xf numFmtId="0" fontId="26" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="general" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="27" fillId="5" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="general" vertical="bottom"/>
+    </xf>
+    <xf numFmtId="0" fontId="28" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="general" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="29" fillId="3" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="30" fillId="4" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="general" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="31" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="general" vertical="bottom"/>
     </xf>
   </cellXfs>
@@ -1031,62 +1099,68 @@
   </cols>
   <sheetData>
     <row r="1" ht="30" customHeight="1" s="14">
-      <c r="A1" s="32" t="inlineStr">
+      <c r="A1" s="42" t="inlineStr">
         <is>
           <t>The Planting Project: Weekly Tracker</t>
         </is>
       </c>
       <c r="B1" s="16" t="n"/>
-      <c r="C1" s="33" t="inlineStr">
+      <c r="C1" s="29" t="inlineStr">
         <is>
           <t>The Pastoral Guide</t>
         </is>
       </c>
     </row>
     <row r="2" ht="16.15" customHeight="1" s="14">
-      <c r="A2" s="34" t="inlineStr">
+      <c r="A2" s="43" t="inlineStr">
         <is>
           <t>How to use this sheet</t>
         </is>
       </c>
     </row>
+    <row r="3"/>
     <row r="4" ht="30" customHeight="1" s="14">
-      <c r="A4" s="35" t="inlineStr">
+      <c r="A4" s="44" t="inlineStr">
         <is>
           <t>•  Each pair has their own tab, labelled Pair 1 to Pair 10; find yours along the bottom.</t>
         </is>
       </c>
     </row>
+    <row r="5"/>
     <row r="6" ht="30" customHeight="1" s="14">
-      <c r="A6" s="35" t="inlineStr">
+      <c r="A6" s="44" t="inlineStr">
         <is>
           <t>•  At the top of your tab, fill in your names, your allocated herb, and the date you planted it.</t>
         </is>
       </c>
     </row>
+    <row r="7"/>
     <row r="8" ht="30" customHeight="1" s="14">
-      <c r="A8" s="35" t="inlineStr">
+      <c r="A8" s="44" t="inlineStr">
         <is>
           <t>•  Every week, add a new row to the log: the date you checked your plant, whether it has germinated, its approximate height, what the leaves look like, any problems you noticed, and what you did about it.</t>
         </is>
       </c>
     </row>
+    <row r="9"/>
     <row r="10" ht="30" customHeight="1" s="14">
-      <c r="A10" s="35" t="inlineStr">
+      <c r="A10" s="44" t="inlineStr">
         <is>
           <t>•  The yellow cells are for you to fill in. The first log row is a worked example; replace it with your own real entry rather than leaving it as a placeholder.</t>
         </is>
       </c>
     </row>
+    <row r="11"/>
     <row r="12" ht="30" customHeight="1" s="14">
-      <c r="A12" s="35" t="inlineStr">
+      <c r="A12" s="44" t="inlineStr">
         <is>
           <t>•  You can add extra rows any week you like; just keep the same columns.</t>
         </is>
       </c>
     </row>
+    <row r="13"/>
     <row r="14" ht="30" customHeight="1" s="14">
-      <c r="A14" s="35" t="inlineStr">
+      <c r="A14" s="44" t="inlineStr">
         <is>
           <t>•  Take a photo each week too, and keep it somewhere safe (e.g. your Google Photos or a shared folder); you’ll want it later for the family cooking challenge writeup.</t>
         </is>
@@ -1119,20 +1193,21 @@
   </cols>
   <sheetData>
     <row r="1" ht="26" customHeight="1" s="14">
-      <c r="A1" s="36" t="inlineStr">
+      <c r="A1" s="45" t="inlineStr">
         <is>
           <t>Pair 9: Herb Log</t>
         </is>
       </c>
-      <c r="F1" s="37" t="inlineStr">
+      <c r="F1" s="31" t="inlineStr">
         <is>
           <t>The Pastoral Guide</t>
         </is>
       </c>
       <c r="G1" s="30" t="n"/>
     </row>
+    <row r="2"/>
     <row r="3" ht="31.5" customHeight="1" s="14">
-      <c r="A3" s="38" t="inlineStr">
+      <c r="A3" s="46" t="inlineStr">
         <is>
           <t>Our names</t>
         </is>
@@ -1142,7 +1217,7 @@
       <c r="D3" s="22" t="n"/>
     </row>
     <row r="4" ht="31.5" customHeight="1" s="14">
-      <c r="A4" s="38" t="inlineStr">
+      <c r="A4" s="46" t="inlineStr">
         <is>
           <t>Our allocated herb</t>
         </is>
@@ -1152,7 +1227,7 @@
       <c r="D4" s="22" t="n"/>
     </row>
     <row r="5" ht="31.5" customHeight="1" s="14">
-      <c r="A5" s="38" t="inlineStr">
+      <c r="A5" s="46" t="inlineStr">
         <is>
           <t>Date planted</t>
         </is>
@@ -1162,7 +1237,7 @@
       <c r="D5" s="22" t="n"/>
     </row>
     <row r="6" ht="31.5" customHeight="1" s="14">
-      <c r="A6" s="38" t="inlineStr">
+      <c r="A6" s="46" t="inlineStr">
         <is>
           <t>Plant’s name (optional)</t>
         </is>
@@ -1172,76 +1247,76 @@
       <c r="D6" s="22" t="n"/>
     </row>
     <row r="7" ht="16.15" customHeight="1" s="14">
-      <c r="A7" s="34" t="inlineStr">
+      <c r="A7" s="43" t="inlineStr">
         <is>
           <t>Weekly log</t>
         </is>
       </c>
     </row>
     <row r="8" ht="27.75" customHeight="1" s="14">
-      <c r="A8" s="39" t="inlineStr">
+      <c r="A8" s="47" t="inlineStr">
         <is>
           <t>Date</t>
         </is>
       </c>
-      <c r="B8" s="39" t="inlineStr">
+      <c r="B8" s="47" t="inlineStr">
         <is>
           <t>Germinated?</t>
         </is>
       </c>
-      <c r="C8" s="39" t="inlineStr">
+      <c r="C8" s="47" t="inlineStr">
         <is>
           <t>Height (cm)</t>
         </is>
       </c>
-      <c r="D8" s="39" t="inlineStr">
+      <c r="D8" s="47" t="inlineStr">
         <is>
           <t>Leaves</t>
         </is>
       </c>
-      <c r="E8" s="39" t="inlineStr">
+      <c r="E8" s="47" t="inlineStr">
         <is>
           <t>Problems noticed</t>
         </is>
       </c>
-      <c r="F8" s="39" t="inlineStr">
+      <c r="F8" s="47" t="inlineStr">
         <is>
           <t>What we did</t>
         </is>
       </c>
     </row>
     <row r="9" ht="30" customHeight="1" s="14">
-      <c r="A9" s="40" t="inlineStr">
+      <c r="A9" s="48" t="inlineStr">
         <is>
           <t>12 Sep 2026</t>
         </is>
       </c>
-      <c r="B9" s="40" t="inlineStr">
+      <c r="B9" s="48" t="inlineStr">
         <is>
           <t>Yes, 4 seedlings</t>
         </is>
       </c>
-      <c r="C9" s="40" t="inlineStr">
+      <c r="C9" s="48" t="inlineStr">
         <is>
           <t>3 cm</t>
         </is>
       </c>
-      <c r="D9" s="40" t="inlineStr">
+      <c r="D9" s="48" t="inlineStr">
         <is>
           <t>First tiny leaves showing</t>
         </is>
       </c>
-      <c r="E9" s="40" t="inlineStr">
+      <c r="E9" s="48" t="inlineStr">
         <is>
           <t>A couple of seeds didn’t sprout</t>
         </is>
       </c>
-      <c r="F9" s="40" t="inlineStr">
+      <c r="F9" s="48" t="inlineStr">
         <is>
           <t>Watered lightly, moved to a sunnier windowsill</t>
         </is>
       </c>
-      <c r="G9" s="41" t="inlineStr">
+      <c r="G9" s="49" t="inlineStr">
         <is>
           <t>← example, replace with your own</t>
         </is>
@@ -1351,20 +1426,21 @@
   </cols>
   <sheetData>
     <row r="1" ht="26" customHeight="1" s="14">
-      <c r="A1" s="36" t="inlineStr">
+      <c r="A1" s="45" t="inlineStr">
         <is>
           <t>Pair 10: Herb Log</t>
         </is>
       </c>
-      <c r="F1" s="37" t="inlineStr">
+      <c r="F1" s="31" t="inlineStr">
         <is>
           <t>The Pastoral Guide</t>
         </is>
       </c>
       <c r="G1" s="30" t="n"/>
     </row>
+    <row r="2"/>
     <row r="3" ht="31.5" customHeight="1" s="14">
-      <c r="A3" s="38" t="inlineStr">
+      <c r="A3" s="46" t="inlineStr">
         <is>
           <t>Our names</t>
         </is>
@@ -1374,7 +1450,7 @@
       <c r="D3" s="22" t="n"/>
     </row>
     <row r="4" ht="31.5" customHeight="1" s="14">
-      <c r="A4" s="38" t="inlineStr">
+      <c r="A4" s="46" t="inlineStr">
         <is>
           <t>Our allocated herb</t>
         </is>
@@ -1384,7 +1460,7 @@
       <c r="D4" s="22" t="n"/>
     </row>
     <row r="5" ht="31.5" customHeight="1" s="14">
-      <c r="A5" s="38" t="inlineStr">
+      <c r="A5" s="46" t="inlineStr">
         <is>
           <t>Date planted</t>
         </is>
@@ -1394,7 +1470,7 @@
       <c r="D5" s="22" t="n"/>
     </row>
     <row r="6" ht="31.5" customHeight="1" s="14">
-      <c r="A6" s="38" t="inlineStr">
+      <c r="A6" s="46" t="inlineStr">
         <is>
           <t>Plant’s name (optional)</t>
         </is>
@@ -1404,76 +1480,76 @@
       <c r="D6" s="22" t="n"/>
     </row>
     <row r="7" ht="16.15" customHeight="1" s="14">
-      <c r="A7" s="34" t="inlineStr">
+      <c r="A7" s="43" t="inlineStr">
         <is>
           <t>Weekly log</t>
         </is>
       </c>
     </row>
     <row r="8" ht="27.75" customHeight="1" s="14">
-      <c r="A8" s="39" t="inlineStr">
+      <c r="A8" s="47" t="inlineStr">
         <is>
           <t>Date</t>
         </is>
       </c>
-      <c r="B8" s="39" t="inlineStr">
+      <c r="B8" s="47" t="inlineStr">
         <is>
           <t>Germinated?</t>
         </is>
       </c>
-      <c r="C8" s="39" t="inlineStr">
+      <c r="C8" s="47" t="inlineStr">
         <is>
           <t>Height (cm)</t>
         </is>
       </c>
-      <c r="D8" s="39" t="inlineStr">
+      <c r="D8" s="47" t="inlineStr">
         <is>
           <t>Leaves</t>
         </is>
       </c>
-      <c r="E8" s="39" t="inlineStr">
+      <c r="E8" s="47" t="inlineStr">
         <is>
           <t>Problems noticed</t>
         </is>
       </c>
-      <c r="F8" s="39" t="inlineStr">
+      <c r="F8" s="47" t="inlineStr">
         <is>
           <t>What we did</t>
         </is>
       </c>
     </row>
     <row r="9" ht="30" customHeight="1" s="14">
-      <c r="A9" s="40" t="inlineStr">
+      <c r="A9" s="48" t="inlineStr">
         <is>
           <t>12 Sep 2026</t>
         </is>
       </c>
-      <c r="B9" s="40" t="inlineStr">
+      <c r="B9" s="48" t="inlineStr">
         <is>
           <t>Yes, 4 seedlings</t>
         </is>
       </c>
-      <c r="C9" s="40" t="inlineStr">
+      <c r="C9" s="48" t="inlineStr">
         <is>
           <t>3 cm</t>
         </is>
       </c>
-      <c r="D9" s="40" t="inlineStr">
+      <c r="D9" s="48" t="inlineStr">
         <is>
           <t>First tiny leaves showing</t>
         </is>
       </c>
-      <c r="E9" s="40" t="inlineStr">
+      <c r="E9" s="48" t="inlineStr">
         <is>
           <t>A couple of seeds didn’t sprout</t>
         </is>
       </c>
-      <c r="F9" s="40" t="inlineStr">
+      <c r="F9" s="48" t="inlineStr">
         <is>
           <t>Watered lightly, moved to a sunnier windowsill</t>
         </is>
       </c>
-      <c r="G9" s="41" t="inlineStr">
+      <c r="G9" s="49" t="inlineStr">
         <is>
           <t>← example, replace with your own</t>
         </is>
@@ -1583,20 +1659,21 @@
   </cols>
   <sheetData>
     <row r="1" ht="26" customHeight="1" s="14">
-      <c r="A1" s="36" t="inlineStr">
+      <c r="A1" s="45" t="inlineStr">
         <is>
           <t>Pair 1: Herb Log</t>
         </is>
       </c>
-      <c r="F1" s="37" t="inlineStr">
+      <c r="F1" s="31" t="inlineStr">
         <is>
           <t>The Pastoral Guide</t>
         </is>
       </c>
       <c r="G1" s="30" t="n"/>
     </row>
+    <row r="2"/>
     <row r="3" ht="31.5" customHeight="1" s="14">
-      <c r="A3" s="38" t="inlineStr">
+      <c r="A3" s="46" t="inlineStr">
         <is>
           <t>Our names</t>
         </is>
@@ -1606,7 +1683,7 @@
       <c r="D3" s="22" t="n"/>
     </row>
     <row r="4" ht="31.5" customHeight="1" s="14">
-      <c r="A4" s="38" t="inlineStr">
+      <c r="A4" s="46" t="inlineStr">
         <is>
           <t>Our allocated herb</t>
         </is>
@@ -1616,7 +1693,7 @@
       <c r="D4" s="22" t="n"/>
     </row>
     <row r="5" ht="31.5" customHeight="1" s="14">
-      <c r="A5" s="38" t="inlineStr">
+      <c r="A5" s="46" t="inlineStr">
         <is>
           <t>Date planted</t>
         </is>
@@ -1626,7 +1703,7 @@
       <c r="D5" s="22" t="n"/>
     </row>
     <row r="6" ht="31.5" customHeight="1" s="14">
-      <c r="A6" s="38" t="inlineStr">
+      <c r="A6" s="46" t="inlineStr">
         <is>
           <t>Plant’s name (optional)</t>
         </is>
@@ -1636,76 +1713,76 @@
       <c r="D6" s="22" t="n"/>
     </row>
     <row r="7" ht="16.15" customHeight="1" s="14">
-      <c r="A7" s="34" t="inlineStr">
+      <c r="A7" s="43" t="inlineStr">
         <is>
           <t>Weekly log</t>
         </is>
       </c>
     </row>
     <row r="8" ht="27.75" customHeight="1" s="14">
-      <c r="A8" s="39" t="inlineStr">
+      <c r="A8" s="47" t="inlineStr">
         <is>
           <t>Date</t>
         </is>
       </c>
-      <c r="B8" s="39" t="inlineStr">
+      <c r="B8" s="47" t="inlineStr">
         <is>
           <t>Germinated?</t>
         </is>
       </c>
-      <c r="C8" s="39" t="inlineStr">
+      <c r="C8" s="47" t="inlineStr">
         <is>
           <t>Height (cm)</t>
         </is>
       </c>
-      <c r="D8" s="39" t="inlineStr">
+      <c r="D8" s="47" t="inlineStr">
         <is>
           <t>Leaves</t>
         </is>
       </c>
-      <c r="E8" s="39" t="inlineStr">
+      <c r="E8" s="47" t="inlineStr">
         <is>
           <t>Problems noticed</t>
         </is>
       </c>
-      <c r="F8" s="39" t="inlineStr">
+      <c r="F8" s="47" t="inlineStr">
         <is>
           <t>What we did</t>
         </is>
       </c>
     </row>
     <row r="9" ht="30" customHeight="1" s="14">
-      <c r="A9" s="40" t="inlineStr">
+      <c r="A9" s="48" t="inlineStr">
         <is>
           <t>12 Sep 2026</t>
         </is>
       </c>
-      <c r="B9" s="40" t="inlineStr">
+      <c r="B9" s="48" t="inlineStr">
         <is>
           <t>Yes, 4 seedlings</t>
         </is>
       </c>
-      <c r="C9" s="40" t="inlineStr">
+      <c r="C9" s="48" t="inlineStr">
         <is>
           <t>3 cm</t>
         </is>
       </c>
-      <c r="D9" s="40" t="inlineStr">
+      <c r="D9" s="48" t="inlineStr">
         <is>
           <t>First tiny leaves showing</t>
         </is>
       </c>
-      <c r="E9" s="40" t="inlineStr">
+      <c r="E9" s="48" t="inlineStr">
         <is>
           <t>A couple of seeds didn’t sprout</t>
         </is>
       </c>
-      <c r="F9" s="40" t="inlineStr">
+      <c r="F9" s="48" t="inlineStr">
         <is>
           <t>Watered lightly, moved to a sunnier windowsill</t>
         </is>
       </c>
-      <c r="G9" s="41" t="inlineStr">
+      <c r="G9" s="49" t="inlineStr">
         <is>
           <t>← example, replace with your own</t>
         </is>
@@ -1815,20 +1892,21 @@
   </cols>
   <sheetData>
     <row r="1" ht="26" customHeight="1" s="14">
-      <c r="A1" s="36" t="inlineStr">
+      <c r="A1" s="45" t="inlineStr">
         <is>
           <t>Pair 2: Herb Log</t>
         </is>
       </c>
-      <c r="F1" s="37" t="inlineStr">
+      <c r="F1" s="31" t="inlineStr">
         <is>
           <t>The Pastoral Guide</t>
         </is>
       </c>
       <c r="G1" s="30" t="n"/>
     </row>
+    <row r="2"/>
     <row r="3" ht="31.5" customHeight="1" s="14">
-      <c r="A3" s="38" t="inlineStr">
+      <c r="A3" s="46" t="inlineStr">
         <is>
           <t>Our names</t>
         </is>
@@ -1838,7 +1916,7 @@
       <c r="D3" s="22" t="n"/>
     </row>
     <row r="4" ht="31.5" customHeight="1" s="14">
-      <c r="A4" s="38" t="inlineStr">
+      <c r="A4" s="46" t="inlineStr">
         <is>
           <t>Our allocated herb</t>
         </is>
@@ -1848,7 +1926,7 @@
       <c r="D4" s="22" t="n"/>
     </row>
     <row r="5" ht="31.5" customHeight="1" s="14">
-      <c r="A5" s="38" t="inlineStr">
+      <c r="A5" s="46" t="inlineStr">
         <is>
           <t>Date planted</t>
         </is>
@@ -1858,7 +1936,7 @@
       <c r="D5" s="22" t="n"/>
     </row>
     <row r="6" ht="31.5" customHeight="1" s="14">
-      <c r="A6" s="38" t="inlineStr">
+      <c r="A6" s="46" t="inlineStr">
         <is>
           <t>Plant’s name (optional)</t>
         </is>
@@ -1868,76 +1946,76 @@
       <c r="D6" s="22" t="n"/>
     </row>
     <row r="7" ht="16.15" customHeight="1" s="14">
-      <c r="A7" s="34" t="inlineStr">
+      <c r="A7" s="43" t="inlineStr">
         <is>
           <t>Weekly log</t>
         </is>
       </c>
     </row>
     <row r="8" ht="27.75" customHeight="1" s="14">
-      <c r="A8" s="39" t="inlineStr">
+      <c r="A8" s="47" t="inlineStr">
         <is>
           <t>Date</t>
         </is>
       </c>
-      <c r="B8" s="39" t="inlineStr">
+      <c r="B8" s="47" t="inlineStr">
         <is>
           <t>Germinated?</t>
         </is>
       </c>
-      <c r="C8" s="39" t="inlineStr">
+      <c r="C8" s="47" t="inlineStr">
         <is>
           <t>Height (cm)</t>
         </is>
       </c>
-      <c r="D8" s="39" t="inlineStr">
+      <c r="D8" s="47" t="inlineStr">
         <is>
           <t>Leaves</t>
         </is>
       </c>
-      <c r="E8" s="39" t="inlineStr">
+      <c r="E8" s="47" t="inlineStr">
         <is>
           <t>Problems noticed</t>
         </is>
       </c>
-      <c r="F8" s="39" t="inlineStr">
+      <c r="F8" s="47" t="inlineStr">
         <is>
           <t>What we did</t>
         </is>
       </c>
     </row>
     <row r="9" ht="30" customHeight="1" s="14">
-      <c r="A9" s="40" t="inlineStr">
+      <c r="A9" s="48" t="inlineStr">
         <is>
           <t>12 Sep 2026</t>
         </is>
       </c>
-      <c r="B9" s="40" t="inlineStr">
+      <c r="B9" s="48" t="inlineStr">
         <is>
           <t>Yes, 4 seedlings</t>
         </is>
       </c>
-      <c r="C9" s="40" t="inlineStr">
+      <c r="C9" s="48" t="inlineStr">
         <is>
           <t>3 cm</t>
         </is>
       </c>
-      <c r="D9" s="40" t="inlineStr">
+      <c r="D9" s="48" t="inlineStr">
         <is>
           <t>First tiny leaves showing</t>
         </is>
       </c>
-      <c r="E9" s="40" t="inlineStr">
+      <c r="E9" s="48" t="inlineStr">
         <is>
           <t>A couple of seeds didn’t sprout</t>
         </is>
       </c>
-      <c r="F9" s="40" t="inlineStr">
+      <c r="F9" s="48" t="inlineStr">
         <is>
           <t>Watered lightly, moved to a sunnier windowsill</t>
         </is>
       </c>
-      <c r="G9" s="41" t="inlineStr">
+      <c r="G9" s="49" t="inlineStr">
         <is>
           <t>← example, replace with your own</t>
         </is>
@@ -2047,20 +2125,21 @@
   </cols>
   <sheetData>
     <row r="1" ht="26" customHeight="1" s="14">
-      <c r="A1" s="36" t="inlineStr">
+      <c r="A1" s="45" t="inlineStr">
         <is>
           <t>Pair 3: Herb Log</t>
         </is>
       </c>
-      <c r="F1" s="37" t="inlineStr">
+      <c r="F1" s="31" t="inlineStr">
         <is>
           <t>The Pastoral Guide</t>
         </is>
       </c>
       <c r="G1" s="30" t="n"/>
     </row>
+    <row r="2"/>
     <row r="3" ht="31.5" customHeight="1" s="14">
-      <c r="A3" s="38" t="inlineStr">
+      <c r="A3" s="46" t="inlineStr">
         <is>
           <t>Our names</t>
         </is>
@@ -2070,7 +2149,7 @@
       <c r="D3" s="22" t="n"/>
     </row>
     <row r="4" ht="31.5" customHeight="1" s="14">
-      <c r="A4" s="38" t="inlineStr">
+      <c r="A4" s="46" t="inlineStr">
         <is>
           <t>Our allocated herb</t>
         </is>
@@ -2080,7 +2159,7 @@
       <c r="D4" s="22" t="n"/>
     </row>
     <row r="5" ht="31.5" customHeight="1" s="14">
-      <c r="A5" s="38" t="inlineStr">
+      <c r="A5" s="46" t="inlineStr">
         <is>
           <t>Date planted</t>
         </is>
@@ -2090,7 +2169,7 @@
       <c r="D5" s="22" t="n"/>
     </row>
     <row r="6" ht="31.5" customHeight="1" s="14">
-      <c r="A6" s="38" t="inlineStr">
+      <c r="A6" s="46" t="inlineStr">
         <is>
           <t>Plant’s name (optional)</t>
         </is>
@@ -2100,76 +2179,76 @@
       <c r="D6" s="22" t="n"/>
     </row>
     <row r="7" ht="16.15" customHeight="1" s="14">
-      <c r="A7" s="34" t="inlineStr">
+      <c r="A7" s="43" t="inlineStr">
         <is>
           <t>Weekly log</t>
         </is>
       </c>
     </row>
     <row r="8" ht="27.75" customHeight="1" s="14">
-      <c r="A8" s="39" t="inlineStr">
+      <c r="A8" s="47" t="inlineStr">
         <is>
           <t>Date</t>
         </is>
       </c>
-      <c r="B8" s="39" t="inlineStr">
+      <c r="B8" s="47" t="inlineStr">
         <is>
           <t>Germinated?</t>
         </is>
       </c>
-      <c r="C8" s="39" t="inlineStr">
+      <c r="C8" s="47" t="inlineStr">
         <is>
           <t>Height (cm)</t>
         </is>
       </c>
-      <c r="D8" s="39" t="inlineStr">
+      <c r="D8" s="47" t="inlineStr">
         <is>
           <t>Leaves</t>
         </is>
       </c>
-      <c r="E8" s="39" t="inlineStr">
+      <c r="E8" s="47" t="inlineStr">
         <is>
           <t>Problems noticed</t>
         </is>
       </c>
-      <c r="F8" s="39" t="inlineStr">
+      <c r="F8" s="47" t="inlineStr">
         <is>
           <t>What we did</t>
         </is>
       </c>
     </row>
     <row r="9" ht="30" customHeight="1" s="14">
-      <c r="A9" s="40" t="inlineStr">
+      <c r="A9" s="48" t="inlineStr">
         <is>
           <t>12 Sep 2026</t>
         </is>
       </c>
-      <c r="B9" s="40" t="inlineStr">
+      <c r="B9" s="48" t="inlineStr">
         <is>
           <t>Yes, 4 seedlings</t>
         </is>
       </c>
-      <c r="C9" s="40" t="inlineStr">
+      <c r="C9" s="48" t="inlineStr">
         <is>
           <t>3 cm</t>
         </is>
       </c>
-      <c r="D9" s="40" t="inlineStr">
+      <c r="D9" s="48" t="inlineStr">
         <is>
           <t>First tiny leaves showing</t>
         </is>
       </c>
-      <c r="E9" s="40" t="inlineStr">
+      <c r="E9" s="48" t="inlineStr">
         <is>
           <t>A couple of seeds didn’t sprout</t>
         </is>
       </c>
-      <c r="F9" s="40" t="inlineStr">
+      <c r="F9" s="48" t="inlineStr">
         <is>
           <t>Watered lightly, moved to a sunnier windowsill</t>
         </is>
       </c>
-      <c r="G9" s="41" t="inlineStr">
+      <c r="G9" s="49" t="inlineStr">
         <is>
           <t>← example, replace with your own</t>
         </is>
@@ -2279,20 +2358,21 @@
   </cols>
   <sheetData>
     <row r="1" ht="26" customHeight="1" s="14">
-      <c r="A1" s="36" t="inlineStr">
+      <c r="A1" s="45" t="inlineStr">
         <is>
           <t>Pair 4: Herb Log</t>
         </is>
       </c>
-      <c r="F1" s="37" t="inlineStr">
+      <c r="F1" s="31" t="inlineStr">
         <is>
           <t>The Pastoral Guide</t>
         </is>
       </c>
       <c r="G1" s="30" t="n"/>
     </row>
+    <row r="2"/>
     <row r="3" ht="31.5" customHeight="1" s="14">
-      <c r="A3" s="38" t="inlineStr">
+      <c r="A3" s="46" t="inlineStr">
         <is>
           <t>Our names</t>
         </is>
@@ -2302,7 +2382,7 @@
       <c r="D3" s="22" t="n"/>
     </row>
     <row r="4" ht="31.5" customHeight="1" s="14">
-      <c r="A4" s="38" t="inlineStr">
+      <c r="A4" s="46" t="inlineStr">
         <is>
           <t>Our allocated herb</t>
         </is>
@@ -2312,7 +2392,7 @@
       <c r="D4" s="22" t="n"/>
     </row>
     <row r="5" ht="31.5" customHeight="1" s="14">
-      <c r="A5" s="38" t="inlineStr">
+      <c r="A5" s="46" t="inlineStr">
         <is>
           <t>Date planted</t>
         </is>
@@ -2322,7 +2402,7 @@
       <c r="D5" s="22" t="n"/>
     </row>
     <row r="6" ht="31.5" customHeight="1" s="14">
-      <c r="A6" s="38" t="inlineStr">
+      <c r="A6" s="46" t="inlineStr">
         <is>
           <t>Plant’s name (optional)</t>
         </is>
@@ -2332,76 +2412,76 @@
       <c r="D6" s="22" t="n"/>
     </row>
     <row r="7" ht="16.15" customHeight="1" s="14">
-      <c r="A7" s="34" t="inlineStr">
+      <c r="A7" s="43" t="inlineStr">
         <is>
           <t>Weekly log</t>
         </is>
       </c>
     </row>
     <row r="8" ht="27.75" customHeight="1" s="14">
-      <c r="A8" s="39" t="inlineStr">
+      <c r="A8" s="47" t="inlineStr">
         <is>
           <t>Date</t>
         </is>
       </c>
-      <c r="B8" s="39" t="inlineStr">
+      <c r="B8" s="47" t="inlineStr">
         <is>
           <t>Germinated?</t>
         </is>
       </c>
-      <c r="C8" s="39" t="inlineStr">
+      <c r="C8" s="47" t="inlineStr">
         <is>
           <t>Height (cm)</t>
         </is>
       </c>
-      <c r="D8" s="39" t="inlineStr">
+      <c r="D8" s="47" t="inlineStr">
         <is>
           <t>Leaves</t>
         </is>
       </c>
-      <c r="E8" s="39" t="inlineStr">
+      <c r="E8" s="47" t="inlineStr">
         <is>
           <t>Problems noticed</t>
         </is>
       </c>
-      <c r="F8" s="39" t="inlineStr">
+      <c r="F8" s="47" t="inlineStr">
         <is>
           <t>What we did</t>
         </is>
       </c>
     </row>
     <row r="9" ht="30" customHeight="1" s="14">
-      <c r="A9" s="40" t="inlineStr">
+      <c r="A9" s="48" t="inlineStr">
         <is>
           <t>12 Sep 2026</t>
         </is>
       </c>
-      <c r="B9" s="40" t="inlineStr">
+      <c r="B9" s="48" t="inlineStr">
         <is>
           <t>Yes, 4 seedlings</t>
         </is>
       </c>
-      <c r="C9" s="40" t="inlineStr">
+      <c r="C9" s="48" t="inlineStr">
         <is>
           <t>3 cm</t>
         </is>
       </c>
-      <c r="D9" s="40" t="inlineStr">
+      <c r="D9" s="48" t="inlineStr">
         <is>
           <t>First tiny leaves showing</t>
         </is>
       </c>
-      <c r="E9" s="40" t="inlineStr">
+      <c r="E9" s="48" t="inlineStr">
         <is>
           <t>A couple of seeds didn’t sprout</t>
         </is>
       </c>
-      <c r="F9" s="40" t="inlineStr">
+      <c r="F9" s="48" t="inlineStr">
         <is>
           <t>Watered lightly, moved to a sunnier windowsill</t>
         </is>
       </c>
-      <c r="G9" s="41" t="inlineStr">
+      <c r="G9" s="49" t="inlineStr">
         <is>
           <t>← example, replace with your own</t>
         </is>
@@ -2511,20 +2591,21 @@
   </cols>
   <sheetData>
     <row r="1" ht="26" customHeight="1" s="14">
-      <c r="A1" s="36" t="inlineStr">
+      <c r="A1" s="45" t="inlineStr">
         <is>
           <t>Pair 5: Herb Log</t>
         </is>
       </c>
-      <c r="F1" s="37" t="inlineStr">
+      <c r="F1" s="31" t="inlineStr">
         <is>
           <t>The Pastoral Guide</t>
         </is>
       </c>
       <c r="G1" s="30" t="n"/>
     </row>
+    <row r="2"/>
     <row r="3" ht="31.5" customHeight="1" s="14">
-      <c r="A3" s="38" t="inlineStr">
+      <c r="A3" s="46" t="inlineStr">
         <is>
           <t>Our names</t>
         </is>
@@ -2534,7 +2615,7 @@
       <c r="D3" s="22" t="n"/>
     </row>
     <row r="4" ht="31.5" customHeight="1" s="14">
-      <c r="A4" s="38" t="inlineStr">
+      <c r="A4" s="46" t="inlineStr">
         <is>
           <t>Our allocated herb</t>
         </is>
@@ -2544,7 +2625,7 @@
       <c r="D4" s="22" t="n"/>
     </row>
     <row r="5" ht="31.5" customHeight="1" s="14">
-      <c r="A5" s="38" t="inlineStr">
+      <c r="A5" s="46" t="inlineStr">
         <is>
           <t>Date planted</t>
         </is>
@@ -2554,7 +2635,7 @@
       <c r="D5" s="22" t="n"/>
     </row>
     <row r="6" ht="31.5" customHeight="1" s="14">
-      <c r="A6" s="38" t="inlineStr">
+      <c r="A6" s="46" t="inlineStr">
         <is>
           <t>Plant’s name (optional)</t>
         </is>
@@ -2564,76 +2645,76 @@
       <c r="D6" s="22" t="n"/>
     </row>
     <row r="7" ht="16.15" customHeight="1" s="14">
-      <c r="A7" s="34" t="inlineStr">
+      <c r="A7" s="43" t="inlineStr">
         <is>
           <t>Weekly log</t>
         </is>
       </c>
     </row>
     <row r="8" ht="27.75" customHeight="1" s="14">
-      <c r="A8" s="39" t="inlineStr">
+      <c r="A8" s="47" t="inlineStr">
         <is>
           <t>Date</t>
         </is>
       </c>
-      <c r="B8" s="39" t="inlineStr">
+      <c r="B8" s="47" t="inlineStr">
         <is>
           <t>Germinated?</t>
         </is>
       </c>
-      <c r="C8" s="39" t="inlineStr">
+      <c r="C8" s="47" t="inlineStr">
         <is>
           <t>Height (cm)</t>
         </is>
       </c>
-      <c r="D8" s="39" t="inlineStr">
+      <c r="D8" s="47" t="inlineStr">
         <is>
           <t>Leaves</t>
         </is>
       </c>
-      <c r="E8" s="39" t="inlineStr">
+      <c r="E8" s="47" t="inlineStr">
         <is>
           <t>Problems noticed</t>
         </is>
       </c>
-      <c r="F8" s="39" t="inlineStr">
+      <c r="F8" s="47" t="inlineStr">
         <is>
           <t>What we did</t>
         </is>
       </c>
     </row>
     <row r="9" ht="30" customHeight="1" s="14">
-      <c r="A9" s="40" t="inlineStr">
+      <c r="A9" s="48" t="inlineStr">
         <is>
           <t>12 Sep 2026</t>
         </is>
       </c>
-      <c r="B9" s="40" t="inlineStr">
+      <c r="B9" s="48" t="inlineStr">
         <is>
           <t>Yes, 4 seedlings</t>
         </is>
       </c>
-      <c r="C9" s="40" t="inlineStr">
+      <c r="C9" s="48" t="inlineStr">
         <is>
           <t>3 cm</t>
         </is>
       </c>
-      <c r="D9" s="40" t="inlineStr">
+      <c r="D9" s="48" t="inlineStr">
         <is>
           <t>First tiny leaves showing</t>
         </is>
       </c>
-      <c r="E9" s="40" t="inlineStr">
+      <c r="E9" s="48" t="inlineStr">
         <is>
           <t>A couple of seeds didn’t sprout</t>
         </is>
       </c>
-      <c r="F9" s="40" t="inlineStr">
+      <c r="F9" s="48" t="inlineStr">
         <is>
           <t>Watered lightly, moved to a sunnier windowsill</t>
         </is>
       </c>
-      <c r="G9" s="41" t="inlineStr">
+      <c r="G9" s="49" t="inlineStr">
         <is>
           <t>← example, replace with your own</t>
         </is>
@@ -2743,20 +2824,21 @@
   </cols>
   <sheetData>
     <row r="1" ht="26" customHeight="1" s="14">
-      <c r="A1" s="36" t="inlineStr">
+      <c r="A1" s="45" t="inlineStr">
         <is>
           <t>Pair 6: Herb Log</t>
         </is>
       </c>
-      <c r="F1" s="37" t="inlineStr">
+      <c r="F1" s="31" t="inlineStr">
         <is>
           <t>The Pastoral Guide</t>
         </is>
       </c>
       <c r="G1" s="30" t="n"/>
     </row>
+    <row r="2"/>
     <row r="3" ht="31.5" customHeight="1" s="14">
-      <c r="A3" s="38" t="inlineStr">
+      <c r="A3" s="46" t="inlineStr">
         <is>
           <t>Our names</t>
         </is>
@@ -2766,7 +2848,7 @@
       <c r="D3" s="22" t="n"/>
     </row>
     <row r="4" ht="31.5" customHeight="1" s="14">
-      <c r="A4" s="38" t="inlineStr">
+      <c r="A4" s="46" t="inlineStr">
         <is>
           <t>Our allocated herb</t>
         </is>
@@ -2776,7 +2858,7 @@
       <c r="D4" s="22" t="n"/>
     </row>
     <row r="5" ht="31.5" customHeight="1" s="14">
-      <c r="A5" s="38" t="inlineStr">
+      <c r="A5" s="46" t="inlineStr">
         <is>
           <t>Date planted</t>
         </is>
@@ -2786,7 +2868,7 @@
       <c r="D5" s="22" t="n"/>
     </row>
     <row r="6" ht="31.5" customHeight="1" s="14">
-      <c r="A6" s="38" t="inlineStr">
+      <c r="A6" s="46" t="inlineStr">
         <is>
           <t>Plant’s name (optional)</t>
         </is>
@@ -2796,76 +2878,76 @@
       <c r="D6" s="22" t="n"/>
     </row>
     <row r="7" ht="16.15" customHeight="1" s="14">
-      <c r="A7" s="34" t="inlineStr">
+      <c r="A7" s="43" t="inlineStr">
         <is>
           <t>Weekly log</t>
         </is>
       </c>
     </row>
     <row r="8" ht="27.75" customHeight="1" s="14">
-      <c r="A8" s="39" t="inlineStr">
+      <c r="A8" s="47" t="inlineStr">
         <is>
           <t>Date</t>
         </is>
       </c>
-      <c r="B8" s="39" t="inlineStr">
+      <c r="B8" s="47" t="inlineStr">
         <is>
           <t>Germinated?</t>
         </is>
       </c>
-      <c r="C8" s="39" t="inlineStr">
+      <c r="C8" s="47" t="inlineStr">
         <is>
           <t>Height (cm)</t>
         </is>
       </c>
-      <c r="D8" s="39" t="inlineStr">
+      <c r="D8" s="47" t="inlineStr">
         <is>
           <t>Leaves</t>
         </is>
       </c>
-      <c r="E8" s="39" t="inlineStr">
+      <c r="E8" s="47" t="inlineStr">
         <is>
           <t>Problems noticed</t>
         </is>
       </c>
-      <c r="F8" s="39" t="inlineStr">
+      <c r="F8" s="47" t="inlineStr">
         <is>
           <t>What we did</t>
         </is>
       </c>
     </row>
     <row r="9" ht="30" customHeight="1" s="14">
-      <c r="A9" s="40" t="inlineStr">
+      <c r="A9" s="48" t="inlineStr">
         <is>
           <t>12 Sep 2026</t>
         </is>
       </c>
-      <c r="B9" s="40" t="inlineStr">
+      <c r="B9" s="48" t="inlineStr">
         <is>
           <t>Yes, 4 seedlings</t>
         </is>
       </c>
-      <c r="C9" s="40" t="inlineStr">
+      <c r="C9" s="48" t="inlineStr">
         <is>
           <t>3 cm</t>
         </is>
       </c>
-      <c r="D9" s="40" t="inlineStr">
+      <c r="D9" s="48" t="inlineStr">
         <is>
           <t>First tiny leaves showing</t>
         </is>
       </c>
-      <c r="E9" s="40" t="inlineStr">
+      <c r="E9" s="48" t="inlineStr">
         <is>
           <t>A couple of seeds didn’t sprout</t>
         </is>
       </c>
-      <c r="F9" s="40" t="inlineStr">
+      <c r="F9" s="48" t="inlineStr">
         <is>
           <t>Watered lightly, moved to a sunnier windowsill</t>
         </is>
       </c>
-      <c r="G9" s="41" t="inlineStr">
+      <c r="G9" s="49" t="inlineStr">
         <is>
           <t>← example, replace with your own</t>
         </is>
@@ -2975,20 +3057,21 @@
   </cols>
   <sheetData>
     <row r="1" ht="26" customHeight="1" s="14">
-      <c r="A1" s="36" t="inlineStr">
+      <c r="A1" s="45" t="inlineStr">
         <is>
           <t>Pair 7: Herb Log</t>
         </is>
       </c>
-      <c r="F1" s="37" t="inlineStr">
+      <c r="F1" s="31" t="inlineStr">
         <is>
           <t>The Pastoral Guide</t>
         </is>
       </c>
       <c r="G1" s="30" t="n"/>
     </row>
+    <row r="2"/>
     <row r="3" ht="31.5" customHeight="1" s="14">
-      <c r="A3" s="38" t="inlineStr">
+      <c r="A3" s="46" t="inlineStr">
         <is>
           <t>Our names</t>
         </is>
@@ -2998,7 +3081,7 @@
       <c r="D3" s="22" t="n"/>
     </row>
     <row r="4" ht="31.5" customHeight="1" s="14">
-      <c r="A4" s="38" t="inlineStr">
+      <c r="A4" s="46" t="inlineStr">
         <is>
           <t>Our allocated herb</t>
         </is>
@@ -3008,7 +3091,7 @@
       <c r="D4" s="22" t="n"/>
     </row>
     <row r="5" ht="31.5" customHeight="1" s="14">
-      <c r="A5" s="38" t="inlineStr">
+      <c r="A5" s="46" t="inlineStr">
         <is>
           <t>Date planted</t>
         </is>
@@ -3018,7 +3101,7 @@
       <c r="D5" s="22" t="n"/>
     </row>
     <row r="6" ht="31.5" customHeight="1" s="14">
-      <c r="A6" s="38" t="inlineStr">
+      <c r="A6" s="46" t="inlineStr">
         <is>
           <t>Plant’s name (optional)</t>
         </is>
@@ -3028,76 +3111,76 @@
       <c r="D6" s="22" t="n"/>
     </row>
     <row r="7" ht="16.15" customHeight="1" s="14">
-      <c r="A7" s="34" t="inlineStr">
+      <c r="A7" s="43" t="inlineStr">
         <is>
           <t>Weekly log</t>
         </is>
       </c>
     </row>
     <row r="8" ht="27.75" customHeight="1" s="14">
-      <c r="A8" s="39" t="inlineStr">
+      <c r="A8" s="47" t="inlineStr">
         <is>
           <t>Date</t>
         </is>
       </c>
-      <c r="B8" s="39" t="inlineStr">
+      <c r="B8" s="47" t="inlineStr">
         <is>
           <t>Germinated?</t>
         </is>
       </c>
-      <c r="C8" s="39" t="inlineStr">
+      <c r="C8" s="47" t="inlineStr">
         <is>
           <t>Height (cm)</t>
         </is>
       </c>
-      <c r="D8" s="39" t="inlineStr">
+      <c r="D8" s="47" t="inlineStr">
         <is>
           <t>Leaves</t>
         </is>
       </c>
-      <c r="E8" s="39" t="inlineStr">
+      <c r="E8" s="47" t="inlineStr">
         <is>
           <t>Problems noticed</t>
         </is>
       </c>
-      <c r="F8" s="39" t="inlineStr">
+      <c r="F8" s="47" t="inlineStr">
         <is>
           <t>What we did</t>
         </is>
       </c>
     </row>
     <row r="9" ht="30" customHeight="1" s="14">
-      <c r="A9" s="40" t="inlineStr">
+      <c r="A9" s="48" t="inlineStr">
         <is>
           <t>12 Sep 2026</t>
         </is>
       </c>
-      <c r="B9" s="40" t="inlineStr">
+      <c r="B9" s="48" t="inlineStr">
         <is>
           <t>Yes, 4 seedlings</t>
         </is>
       </c>
-      <c r="C9" s="40" t="inlineStr">
+      <c r="C9" s="48" t="inlineStr">
         <is>
           <t>3 cm</t>
         </is>
       </c>
-      <c r="D9" s="40" t="inlineStr">
+      <c r="D9" s="48" t="inlineStr">
         <is>
           <t>First tiny leaves showing</t>
         </is>
       </c>
-      <c r="E9" s="40" t="inlineStr">
+      <c r="E9" s="48" t="inlineStr">
         <is>
           <t>A couple of seeds didn’t sprout</t>
         </is>
       </c>
-      <c r="F9" s="40" t="inlineStr">
+      <c r="F9" s="48" t="inlineStr">
         <is>
           <t>Watered lightly, moved to a sunnier windowsill</t>
         </is>
       </c>
-      <c r="G9" s="41" t="inlineStr">
+      <c r="G9" s="49" t="inlineStr">
         <is>
           <t>← example, replace with your own</t>
         </is>
@@ -3207,20 +3290,21 @@
   </cols>
   <sheetData>
     <row r="1" ht="26" customHeight="1" s="14">
-      <c r="A1" s="36" t="inlineStr">
+      <c r="A1" s="45" t="inlineStr">
         <is>
           <t>Pair 8: Herb Log</t>
         </is>
       </c>
-      <c r="F1" s="37" t="inlineStr">
+      <c r="F1" s="31" t="inlineStr">
         <is>
           <t>The Pastoral Guide</t>
         </is>
       </c>
       <c r="G1" s="30" t="n"/>
     </row>
+    <row r="2"/>
     <row r="3" ht="31.5" customHeight="1" s="14">
-      <c r="A3" s="38" t="inlineStr">
+      <c r="A3" s="46" t="inlineStr">
         <is>
           <t>Our names</t>
         </is>
@@ -3230,7 +3314,7 @@
       <c r="D3" s="22" t="n"/>
     </row>
     <row r="4" ht="31.5" customHeight="1" s="14">
-      <c r="A4" s="38" t="inlineStr">
+      <c r="A4" s="46" t="inlineStr">
         <is>
           <t>Our allocated herb</t>
         </is>
@@ -3240,7 +3324,7 @@
       <c r="D4" s="22" t="n"/>
     </row>
     <row r="5" ht="31.5" customHeight="1" s="14">
-      <c r="A5" s="38" t="inlineStr">
+      <c r="A5" s="46" t="inlineStr">
         <is>
           <t>Date planted</t>
         </is>
@@ -3250,7 +3334,7 @@
       <c r="D5" s="22" t="n"/>
     </row>
     <row r="6" ht="31.5" customHeight="1" s="14">
-      <c r="A6" s="38" t="inlineStr">
+      <c r="A6" s="46" t="inlineStr">
         <is>
           <t>Plant’s name (optional)</t>
         </is>
@@ -3260,76 +3344,76 @@
       <c r="D6" s="22" t="n"/>
     </row>
     <row r="7" ht="16.15" customHeight="1" s="14">
-      <c r="A7" s="34" t="inlineStr">
+      <c r="A7" s="43" t="inlineStr">
         <is>
           <t>Weekly log</t>
         </is>
       </c>
     </row>
     <row r="8" ht="27.75" customHeight="1" s="14">
-      <c r="A8" s="39" t="inlineStr">
+      <c r="A8" s="47" t="inlineStr">
         <is>
           <t>Date</t>
         </is>
       </c>
-      <c r="B8" s="39" t="inlineStr">
+      <c r="B8" s="47" t="inlineStr">
         <is>
           <t>Germinated?</t>
         </is>
       </c>
-      <c r="C8" s="39" t="inlineStr">
+      <c r="C8" s="47" t="inlineStr">
         <is>
           <t>Height (cm)</t>
         </is>
       </c>
-      <c r="D8" s="39" t="inlineStr">
+      <c r="D8" s="47" t="inlineStr">
         <is>
           <t>Leaves</t>
         </is>
       </c>
-      <c r="E8" s="39" t="inlineStr">
+      <c r="E8" s="47" t="inlineStr">
         <is>
           <t>Problems noticed</t>
         </is>
       </c>
-      <c r="F8" s="39" t="inlineStr">
+      <c r="F8" s="47" t="inlineStr">
         <is>
           <t>What we did</t>
         </is>
       </c>
     </row>
     <row r="9" ht="30" customHeight="1" s="14">
-      <c r="A9" s="40" t="inlineStr">
+      <c r="A9" s="48" t="inlineStr">
         <is>
           <t>12 Sep 2026</t>
         </is>
       </c>
-      <c r="B9" s="40" t="inlineStr">
+      <c r="B9" s="48" t="inlineStr">
         <is>
           <t>Yes, 4 seedlings</t>
         </is>
       </c>
-      <c r="C9" s="40" t="inlineStr">
+      <c r="C9" s="48" t="inlineStr">
         <is>
           <t>3 cm</t>
         </is>
       </c>
-      <c r="D9" s="40" t="inlineStr">
+      <c r="D9" s="48" t="inlineStr">
         <is>
           <t>First tiny leaves showing</t>
         </is>
       </c>
-      <c r="E9" s="40" t="inlineStr">
+      <c r="E9" s="48" t="inlineStr">
         <is>
           <t>A couple of seeds didn’t sprout</t>
         </is>
       </c>
-      <c r="F9" s="40" t="inlineStr">
+      <c r="F9" s="48" t="inlineStr">
         <is>
           <t>Watered lightly, moved to a sunnier windowsill</t>
         </is>
       </c>
-      <c r="G9" s="41" t="inlineStr">
+      <c r="G9" s="49" t="inlineStr">
         <is>
           <t>← example, replace with your own</t>
         </is>

</xml_diff>